<commit_message>
Run exp1: regenerate plots and table
</commit_message>
<xml_diff>
--- a/lab1/data/实验1数据.xlsx
+++ b/lab1/data/实验1数据.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\siriuschen\lab\lab1\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21621C7D-410E-45DA-8435-387885CF52EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14FDAC7-2A00-4B0F-9464-0FF297F2C0EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,11 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <t>工作状态/参数名称</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>n1/%</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -143,10 +139,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -431,59 +430,62 @@
   <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="C1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
       <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>13</v>
-      </c>
-      <c r="P1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
+        <v>15</v>
+      </c>
+      <c r="B2">
+        <v>13</v>
       </c>
       <c r="C2">
         <v>72.53</v>
@@ -529,7 +531,9 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B3" s="1"/>
+      <c r="B3">
+        <v>18.09</v>
+      </c>
       <c r="C3">
         <v>75.510000000000005</v>
       </c>
@@ -574,7 +578,9 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B4" s="1"/>
+      <c r="B4">
+        <v>26.85</v>
+      </c>
       <c r="C4">
         <v>80.349999999999994</v>
       </c>
@@ -619,7 +625,9 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B5" s="1"/>
+      <c r="B5">
+        <v>35.47</v>
+      </c>
       <c r="C5">
         <v>85.14</v>
       </c>
@@ -664,7 +672,9 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B6" s="1"/>
+      <c r="B6">
+        <v>44.19</v>
+      </c>
       <c r="C6">
         <v>90.19</v>
       </c>
@@ -709,7 +719,9 @@
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B7" s="1"/>
+      <c r="B7">
+        <v>54.51</v>
+      </c>
       <c r="C7">
         <v>95.26</v>
       </c>
@@ -754,7 +766,9 @@
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B8" s="1"/>
+      <c r="B8">
+        <v>58.98</v>
+      </c>
       <c r="C8">
         <v>97.08</v>
       </c>
@@ -800,9 +814,11 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="1"/>
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>80</v>
+      </c>
       <c r="C9">
         <v>99.86</v>
       </c>
@@ -848,13 +864,13 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="B10">
+        <v>83.19</v>
+      </c>
       <c r="C10">
-        <v>83.19</v>
+        <v>99.87</v>
       </c>
       <c r="D10">
         <v>97.89</v>
@@ -898,9 +914,11 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
+      <c r="B11">
+        <v>88.85</v>
+      </c>
       <c r="C11">
-        <v>88.85</v>
+        <v>99.86</v>
       </c>
       <c r="D11">
         <v>97.89</v>
@@ -944,9 +962,11 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
+      <c r="B12">
+        <v>99.63</v>
+      </c>
       <c r="C12">
-        <v>99.63</v>
+        <v>99.84</v>
       </c>
       <c r="D12">
         <v>97.9</v>
@@ -990,9 +1010,11 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
+      <c r="B13">
+        <v>107.99</v>
+      </c>
       <c r="C13">
-        <v>107.99</v>
+        <v>99.84</v>
       </c>
       <c r="D13">
         <v>97.89</v>
@@ -1036,9 +1058,11 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
+      <c r="B14">
+        <v>114.72</v>
+      </c>
       <c r="C14">
-        <v>114.72</v>
+        <v>99.84</v>
       </c>
       <c r="D14">
         <v>97.9</v>
@@ -1081,9 +1105,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B2:B9"/>
-    <mergeCell ref="B10:B14"/>
+  <mergeCells count="1">
     <mergeCell ref="A10:A14"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>